<commit_message>
Ireland Testcase New added
</commit_message>
<xml_diff>
--- a/Data/Workday_NewHire_Ireland_PK4_APUpdated.xlsx
+++ b/Data/Workday_NewHire_Ireland_PK4_APUpdated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\WorkdaySuite_Playwright_GP_Ireland\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78C1B6D-F48A-4887-B13E-8209F080F5C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E666D7F4-090D-4451-86A3-242D32DF2EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="528" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="528" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Information" sheetId="42" r:id="rId1"/>
@@ -326,7 +326,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5159" uniqueCount="1479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5174" uniqueCount="1494">
   <si>
     <t>Version</t>
   </si>
@@ -4903,6 +4903,51 @@
   </si>
   <si>
     <t>2576979JA</t>
+  </si>
+  <si>
+    <t>2576988JA</t>
+  </si>
+  <si>
+    <t>2576989JA</t>
+  </si>
+  <si>
+    <t>2576990JA</t>
+  </si>
+  <si>
+    <t>2576991JA</t>
+  </si>
+  <si>
+    <t>2576992JA</t>
+  </si>
+  <si>
+    <t>2576993JA</t>
+  </si>
+  <si>
+    <t>2576994JA</t>
+  </si>
+  <si>
+    <t>2576995JA</t>
+  </si>
+  <si>
+    <t>2576996JA</t>
+  </si>
+  <si>
+    <t>2576997JA</t>
+  </si>
+  <si>
+    <t>2576998JA</t>
+  </si>
+  <si>
+    <t>2576999JA</t>
+  </si>
+  <si>
+    <t>2577000JA</t>
+  </si>
+  <si>
+    <t>2577001JA</t>
+  </si>
+  <si>
+    <t>2577002JA</t>
   </si>
 </sst>
 </file>
@@ -5901,7 +5946,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="237">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -6455,6 +6500,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6813,22 +6859,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="230" t="s">
+      <c r="A1" s="231" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="231"/>
-      <c r="C1" s="232"/>
-      <c r="F1" s="230" t="s">
+      <c r="B1" s="232"/>
+      <c r="C1" s="233"/>
+      <c r="F1" s="231" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="232"/>
+      <c r="G1" s="233"/>
     </row>
     <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="233"/>
-      <c r="B2" s="234"/>
-      <c r="C2" s="235"/>
-      <c r="F2" s="233"/>
-      <c r="G2" s="235"/>
+      <c r="A2" s="234"/>
+      <c r="B2" s="235"/>
+      <c r="C2" s="236"/>
+      <c r="F2" s="234"/>
+      <c r="G2" s="236"/>
     </row>
     <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="1:7" ht="19" thickBot="1" x14ac:dyDescent="0.5">
@@ -7690,7 +7736,7 @@
       </c>
       <c r="J2" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY())&lt;10,"0"&amp;MONTH(TODAY())&amp;"/",MONTH(TODAY())&amp;"/") &amp; IF(DAY(TODAY())&lt;10,"0"&amp;DAY(TODAY())&amp;"/",DAY(TODAY())&amp;"/") &amp; YEAR(TODAY())</f>
-        <v>04/04/2025</v>
+        <v>04/08/2025</v>
       </c>
       <c r="K2" s="29" t="s">
         <v>30</v>
@@ -7715,7 +7761,7 @@
       </c>
       <c r="R2" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY())&lt;10,"0"&amp;MONTH(TODAY())&amp;"/",MONTH(TODAY())&amp;"/") &amp; IF(DAY(TODAY())&lt;10,"0"&amp;DAY(TODAY())&amp;"/",DAY(TODAY())&amp;"/") &amp; YEAR(TODAY())</f>
-        <v>04/04/2025</v>
+        <v>04/08/2025</v>
       </c>
       <c r="S2" s="29" t="s">
         <v>243</v>
@@ -7740,7 +7786,7 @@
       </c>
       <c r="Z2" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY())&lt;10,"0"&amp;MONTH(TODAY())&amp;"/",MONTH(TODAY())&amp;"/") &amp; IF(DAY(TODAY())&lt;10,"0"&amp;DAY(TODAY())&amp;"/",DAY(TODAY())&amp;"/") &amp; YEAR(TODAY())</f>
-        <v>04/04/2025</v>
+        <v>04/08/2025</v>
       </c>
       <c r="AA2" t="s">
         <v>151</v>
@@ -7771,7 +7817,7 @@
       </c>
       <c r="AO2" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+100)&lt;10,"0"&amp;MONTH(TODAY()+100)&amp;"/",MONTH(TODAY()+100)&amp;"/") &amp; IF(DAY(TODAY()+100)&lt;10,"0"&amp;DAY(TODAY()+100)&amp;"/",DAY(TODAY()+100)&amp;"/") &amp; YEAR(TODAY()+100)</f>
-        <v>07/13/2025</v>
+        <v>07/17/2025</v>
       </c>
       <c r="AP2" t="s">
         <v>234</v>
@@ -7831,7 +7877,7 @@
       </c>
       <c r="J3" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()-10)&lt;10,"0"&amp;MONTH(TODAY()-10)&amp;"/",MONTH(TODAY()-10))&amp;"/" &amp; IF(DAY(TODAY()-10)&lt;10,"0"&amp;DAY(TODAY()-10)&amp;"/",DAY(TODAY()-10)&amp;"/") &amp; YEAR(TODAY()-10)</f>
-        <v>03//25/2025</v>
+        <v>03//29/2025</v>
       </c>
       <c r="L3" s="29" t="s">
         <v>258</v>
@@ -7851,7 +7897,7 @@
       </c>
       <c r="R3" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+100)&lt;10,"0"&amp;MONTH(TODAY()+100)&amp;"/",MONTH(TODAY()+100)&amp;"/") &amp; IF(DAY(TODAY()+100)&lt;10,"0"&amp;DAY(TODAY()+100)&amp;"/",DAY(TODAY()+100)&amp;"/") &amp; YEAR(TODAY()+100)</f>
-        <v>07/13/2025</v>
+        <v>07/17/2025</v>
       </c>
       <c r="T3" s="29" t="s">
         <v>156</v>
@@ -7873,7 +7919,7 @@
       </c>
       <c r="Z3" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+100)&lt;10,"0"&amp;MONTH(TODAY()+100)&amp;"/",MONTH(TODAY()+100)&amp;"/") &amp; IF(DAY(TODAY()+100)&lt;10,"0"&amp;DAY(TODAY()+100)&amp;"/",DAY(TODAY()+100)&amp;"/") &amp; YEAR(TODAY()+100)</f>
-        <v>07/13/2025</v>
+        <v>07/17/2025</v>
       </c>
       <c r="AA3" s="34"/>
       <c r="AB3" s="34"/>
@@ -7905,7 +7951,7 @@
       </c>
       <c r="AO3" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+1000)&lt;10,"0"&amp;MONTH(TODAY()+1000)&amp;"/",MONTH(TODAY()+1000)&amp;"/") &amp; IF(DAY(TODAY()+1000)&lt;10,"0"&amp;DAY(TODAY()+1000)&amp;"/",DAY(TODAY()+1000)&amp;"/") &amp; YEAR(TODAY()+1000)</f>
-        <v>12/30/2027</v>
+        <v>01/03/2028</v>
       </c>
       <c r="AP3" t="s">
         <v>36</v>
@@ -7931,7 +7977,7 @@
       </c>
       <c r="J4" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+10)&lt;10,"0"&amp;MONTH(TODAY()+10)&amp;"/",MONTH(TODAY()+10)&amp;"/") &amp; IF(DAY(TODAY()+10)&lt;10,"0"&amp;DAY(TODAY()+10)&amp;"/",DAY(TODAY()+10)&amp;"/") &amp; YEAR(TODAY()+10)</f>
-        <v>04/14/2025</v>
+        <v>04/18/2025</v>
       </c>
       <c r="L4" s="29" t="s">
         <v>272</v>
@@ -7947,7 +7993,7 @@
       </c>
       <c r="R4" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+1000)&lt;10,"0"&amp;MONTH(TODAY()+1000)&amp;"/",MONTH(TODAY()+1000)&amp;"/") &amp; IF(DAY(TODAY()+1000)&lt;10,"0"&amp;DAY(TODAY()+1000)&amp;"/",DAY(TODAY()+1000)&amp;"/") &amp; YEAR(TODAY()+1000)</f>
-        <v>12/30/2027</v>
+        <v>01/03/2028</v>
       </c>
       <c r="W4" s="29" t="s">
         <v>273</v>
@@ -7960,7 +8006,7 @@
       </c>
       <c r="Z4" s="34" t="str">
         <f ca="1">IF(MONTH(TODAY()+1000)&lt;10,"0"&amp;MONTH(TODAY()+1000)&amp;"/",MONTH(TODAY()+1000)&amp;"/") &amp; IF(DAY(TODAY()+1000)&lt;10,"0"&amp;DAY(TODAY()+1000)&amp;"/",DAY(TODAY()+1000)&amp;"/") &amp; YEAR(TODAY()+1000)</f>
-        <v>12/30/2027</v>
+        <v>01/03/2028</v>
       </c>
       <c r="AA4" s="34"/>
       <c r="AB4" s="34"/>
@@ -32654,63 +32700,63 @@
       <c r="F25" s="186"/>
       <c r="G25" s="200">
         <f ca="1">TODAY()-31</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="H25" s="200">
         <f t="shared" ref="H25:U25" ca="1" si="2">TODAY()-31</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="I25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="J25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="K25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="L25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="M25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="N25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="O25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="P25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="Q25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="R25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="S25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="T25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="U25" s="200">
         <f t="shared" ca="1" si="2"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="26" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -33451,63 +33497,63 @@
       <c r="F37" s="186"/>
       <c r="G37" s="211">
         <f ca="1">G25</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="H37" s="211">
         <f ca="1">H25</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="I37" s="211">
         <f ca="1">I25</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="J37" s="211">
         <f ca="1">J25</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="K37" s="211">
         <f ca="1">K25</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="L37" s="211">
         <f t="shared" ref="L37:U37" ca="1" si="3">L25</f>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="M37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="N37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="O37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="P37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="Q37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="R37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="S37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="T37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
       <c r="U37" s="211">
         <f t="shared" ca="1" si="3"/>
-        <v>45720</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="38" spans="1:21" s="29" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -33531,63 +33577,63 @@
       <c r="F38" s="186"/>
       <c r="G38" s="200">
         <f ca="1">G37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="H38" s="200">
         <f ca="1">H37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="I38" s="200">
         <f ca="1">I37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="J38" s="200">
         <f ca="1">J37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="K38" s="200">
         <f ca="1">K37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="L38" s="200">
         <f t="shared" ref="L38:U38" ca="1" si="4">L37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="M38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="N38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="O38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="P38" s="200">
         <f ca="1">P37+90</f>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="Q38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="R38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="S38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="T38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
       <c r="U38" s="200">
         <f t="shared" ca="1" si="4"/>
-        <v>45810</v>
+        <v>45814</v>
       </c>
     </row>
     <row r="39" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -34270,14 +34316,14 @@
       </c>
       <c r="H49" s="207">
         <f ca="1">H37+365</f>
-        <v>46085</v>
+        <v>46089</v>
       </c>
       <c r="I49" s="207" t="s">
         <v>73</v>
       </c>
       <c r="J49" s="207">
         <f ca="1">J37+365</f>
-        <v>46085</v>
+        <v>46089</v>
       </c>
       <c r="K49" s="207" t="s">
         <v>73</v>
@@ -34290,28 +34336,28 @@
       </c>
       <c r="N49" s="207">
         <f ca="1">N37+365</f>
-        <v>46085</v>
+        <v>46089</v>
       </c>
       <c r="O49" s="207" t="s">
         <v>73</v>
       </c>
       <c r="P49" s="207">
         <f ca="1">P37+365</f>
-        <v>46085</v>
+        <v>46089</v>
       </c>
       <c r="Q49" s="207" t="s">
         <v>73</v>
       </c>
       <c r="R49" s="207">
         <f ca="1">R37+365</f>
-        <v>46085</v>
+        <v>46089</v>
       </c>
       <c r="S49" s="207" t="s">
         <v>73</v>
       </c>
       <c r="T49" s="207">
         <f ca="1">T37+365</f>
-        <v>46085</v>
+        <v>46089</v>
       </c>
       <c r="U49" s="207" t="s">
         <v>73</v>
@@ -38053,7 +38099,7 @@
         <v>2576987JA</v>
       </c>
     </row>
-    <row r="145" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C145" s="218">
         <v>2576988</v>
       </c>
@@ -38064,8 +38110,11 @@
         <f t="shared" si="3"/>
         <v>2576988JA</v>
       </c>
-    </row>
-    <row r="146" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G145" s="29" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="146" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C146" s="218">
         <v>2576989</v>
       </c>
@@ -38076,8 +38125,11 @@
         <f t="shared" si="3"/>
         <v>2576989JA</v>
       </c>
-    </row>
-    <row r="147" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G146" s="29" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="147" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C147" s="218">
         <v>2576990</v>
       </c>
@@ -38088,8 +38140,11 @@
         <f t="shared" si="3"/>
         <v>2576990JA</v>
       </c>
-    </row>
-    <row r="148" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G147" s="29" t="s">
+        <v>1481</v>
+      </c>
+    </row>
+    <row r="148" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C148" s="218">
         <v>2576991</v>
       </c>
@@ -38100,8 +38155,11 @@
         <f t="shared" si="3"/>
         <v>2576991JA</v>
       </c>
-    </row>
-    <row r="149" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G148" s="29" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="149" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C149" s="218">
         <v>2576992</v>
       </c>
@@ -38112,8 +38170,11 @@
         <f t="shared" si="3"/>
         <v>2576992JA</v>
       </c>
-    </row>
-    <row r="150" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G149" s="29" t="s">
+        <v>1483</v>
+      </c>
+    </row>
+    <row r="150" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C150" s="218">
         <v>2576993</v>
       </c>
@@ -38124,8 +38185,11 @@
         <f t="shared" si="3"/>
         <v>2576993JA</v>
       </c>
-    </row>
-    <row r="151" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G150" s="29" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="151" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C151" s="218">
         <v>2576994</v>
       </c>
@@ -38136,8 +38200,11 @@
         <f t="shared" si="3"/>
         <v>2576994JA</v>
       </c>
-    </row>
-    <row r="152" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G151" s="29" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="152" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C152" s="218">
         <v>2576995</v>
       </c>
@@ -38148,8 +38215,11 @@
         <f t="shared" si="3"/>
         <v>2576995JA</v>
       </c>
-    </row>
-    <row r="153" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G152" s="29" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="153" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C153" s="218">
         <v>2576996</v>
       </c>
@@ -38160,8 +38230,11 @@
         <f t="shared" si="3"/>
         <v>2576996JA</v>
       </c>
-    </row>
-    <row r="154" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G153" s="29" t="s">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="154" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C154" s="218">
         <v>2576997</v>
       </c>
@@ -38172,8 +38245,11 @@
         <f t="shared" si="3"/>
         <v>2576997JA</v>
       </c>
-    </row>
-    <row r="155" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G154" s="29" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="155" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C155" s="218">
         <v>2576998</v>
       </c>
@@ -38184,8 +38260,11 @@
         <f t="shared" si="3"/>
         <v>2576998JA</v>
       </c>
-    </row>
-    <row r="156" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G155" s="29" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="156" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C156" s="218">
         <v>2576999</v>
       </c>
@@ -38196,8 +38275,11 @@
         <f t="shared" si="3"/>
         <v>2576999JA</v>
       </c>
-    </row>
-    <row r="157" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G156" s="29" t="s">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="157" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C157" s="218">
         <v>2577000</v>
       </c>
@@ -38208,8 +38290,11 @@
         <f t="shared" si="3"/>
         <v>2577000JA</v>
       </c>
-    </row>
-    <row r="158" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G157" s="29" t="s">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="158" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C158" s="218">
         <v>2577001</v>
       </c>
@@ -38220,8 +38305,11 @@
         <f t="shared" si="3"/>
         <v>2577001JA</v>
       </c>
-    </row>
-    <row r="159" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G158" s="29" t="s">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="159" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C159" s="218">
         <v>2577002</v>
       </c>
@@ -38232,8 +38320,14 @@
         <f t="shared" si="3"/>
         <v>2577002JA</v>
       </c>
-    </row>
-    <row r="160" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="G159" s="29" t="s">
+        <v>1493</v>
+      </c>
+      <c r="H159" s="230">
+        <v>776324</v>
+      </c>
+    </row>
+    <row r="160" spans="3:8" x14ac:dyDescent="0.35">
       <c r="C160" s="218">
         <v>2577003</v>
       </c>
@@ -41125,6 +41219,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001C28CCD5E0F01447929BAFF142255314" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9e105077c73185890e2978400d6c0c32">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="33b4a496-69c9-4eda-b8b7-f258e20f99d0" xmlns:ns4="c5ced6a3-cb0b-445c-8402-1bc366deee8c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0772d52c450de531841c9d1ff9ec7d89" ns3:_="" ns4:_="">
     <xsd:import namespace="33b4a496-69c9-4eda-b8b7-f258e20f99d0"/>
@@ -41347,7 +41447,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -41356,13 +41456,24 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06B61484-8E96-4333-AEC2-06329464E92F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c5ced6a3-cb0b-445c-8402-1bc366deee8c"/>
+    <ds:schemaRef ds:uri="33b4a496-69c9-4eda-b8b7-f258e20f99d0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0725B27-3330-4D57-81C7-C2CB4273E427}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41381,27 +41492,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1499BE8-39AF-4509-A663-6F591C3DD2CC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06B61484-8E96-4333-AEC2-06329464E92F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c5ced6a3-cb0b-445c-8402-1bc366deee8c"/>
-    <ds:schemaRef ds:uri="33b4a496-69c9-4eda-b8b7-f258e20f99d0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>